<commit_message>
Day B deload session logged; sitewide link audit closed out with the wrong-domain related-post link fixed and the hidden sidebar bug cleared sitewide via a single Customizer setting instead of per-post edits
</commit_message>
<xml_diff>
--- a/outputs/website-redesign/2026-09-03-link-audit.xlsx
+++ b/outputs/website-redesign/2026-09-03-link-audit.xlsx
@@ -1106,7 +1106,7 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed 2026-09-03 — edited the link in the block editor (WP REST search API located the exact post: "How to Accelerate Business Growth When the Economy Feels Uncertain," post 11954), replaced the production href with the staging URL via the link-edit popover, saved. Verified live: all 5 instances of this related-article link on the page now resolve to staging.</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1230,6 +1230,14 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Fixed 2026-09-03 — two-part fix. (1) The 7 non-blog pages (Work With Me, The Messy Middle, Mastermind for the Messy Middle, Seven Figure Forum, both Apply pages, Schedule a Conversation) each had their GeneratePress "Sidebar Layout" page setting switched from the default to "No Sidebars" individually, matching how Home/About were already set — the standard classic-metabox-needs-requestMetaBoxUpdates() fix documented elsewhere in this project. (2) All 563 blog posts were fixed in one shot, without touching any individual post: Customizer &gt; Layout &gt; Sidebars &gt; "Single Post Sidebar Layout" was switched from "Content / Sidebar" to "Content (no sidebars)" and published — since no individual post overrides this site-wide default, it applies everywhere at once. Verified: the sidebar div and its ~535 links are now absent from the raw HTML (not just CSS-hidden) on all 7 pages plus a 3-post sample (including the post used in fix #1). No visual regression on any page checked.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>